<commit_message>
changes fix for data
</commit_message>
<xml_diff>
--- a/newui_Greyform/PBU_TERRAHL2(final).xlsx
+++ b/newui_Greyform/PBU_TERRAHL2(final).xlsx
@@ -1557,7 +1557,7 @@
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="Q22" t="n">
         <v>0</v>
@@ -1607,7 +1607,7 @@
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="Q23" t="n">
         <v>0</v>
@@ -1657,7 +1657,7 @@
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="n">
-        <v>-100</v>
+        <v>800</v>
       </c>
       <c r="Q24" t="n">
         <v>0</v>
@@ -1707,7 +1707,7 @@
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="n">
-        <v>-100</v>
+        <v>800</v>
       </c>
       <c r="Q25" t="n">
         <v>0</v>
@@ -1757,7 +1757,7 @@
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="n">
-        <v>-700</v>
+        <v>200</v>
       </c>
       <c r="Q26" t="n">
         <v>0</v>
@@ -1807,7 +1807,7 @@
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="n">
-        <v>-700</v>
+        <v>200</v>
       </c>
       <c r="Q27" t="n">
         <v>0</v>
@@ -1857,7 +1857,7 @@
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="n">
-        <v>-1200</v>
+        <v>-300</v>
       </c>
       <c r="Q28" t="n">
         <v>0</v>
@@ -1907,7 +1907,7 @@
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="n">
-        <v>-1200</v>
+        <v>-300</v>
       </c>
       <c r="Q29" t="n">
         <v>0</v>
@@ -1957,7 +1957,7 @@
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="n">
-        <v>-1200</v>
+        <v>-300</v>
       </c>
       <c r="Q30" t="n">
         <v>0</v>
@@ -2007,7 +2007,7 @@
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="n">
-        <v>-1200</v>
+        <v>-300</v>
       </c>
       <c r="Q31" t="n">
         <v>0</v>
@@ -2039,8 +2039,14 @@
       <c r="H32" t="n">
         <v>1</v>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>blank</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>1</v>
+      </c>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="n">
         <v>1200</v>
@@ -2051,7 +2057,7 @@
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="n">
-        <v>-950</v>
+        <v>-50</v>
       </c>
       <c r="Q32" t="n">
         <v>0</v>
@@ -2083,8 +2089,14 @@
       <c r="H33" t="n">
         <v>1</v>
       </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>blank</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>1</v>
+      </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="n">
         <v>1200</v>
@@ -2095,7 +2107,7 @@
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="n">
-        <v>-950</v>
+        <v>-50</v>
       </c>
       <c r="Q33" t="n">
         <v>0</v>
@@ -2745,10 +2757,10 @@
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="n">
-        <v>-1200</v>
+        <v>-300</v>
       </c>
       <c r="Q46" t="n">
-        <v>0</v>
+        <v>-1800</v>
       </c>
       <c r="R46" t="n">
         <v>-775</v>
@@ -2795,10 +2807,10 @@
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="n">
-        <v>-1200</v>
+        <v>-300</v>
       </c>
       <c r="Q47" t="n">
-        <v>0</v>
+        <v>-1800</v>
       </c>
       <c r="R47" t="n">
         <v>-175</v>
@@ -2845,10 +2857,10 @@
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="n">
-        <v>-1200</v>
+        <v>-300</v>
       </c>
       <c r="Q48" t="n">
-        <v>0</v>
+        <v>-1800</v>
       </c>
       <c r="R48" t="n">
         <v>425</v>
@@ -2895,10 +2907,10 @@
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="n">
-        <v>-1200</v>
+        <v>-300</v>
       </c>
       <c r="Q49" t="n">
-        <v>0</v>
+        <v>-1800</v>
       </c>
       <c r="R49" t="n">
         <v>1025</v>
@@ -2945,10 +2957,10 @@
       <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="n">
-        <v>-1585</v>
+        <v>-685</v>
       </c>
       <c r="Q50" t="n">
-        <v>0</v>
+        <v>-1800</v>
       </c>
       <c r="R50" t="n">
         <v>-775</v>
@@ -2995,10 +3007,10 @@
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="n">
-        <v>-1585</v>
+        <v>-685</v>
       </c>
       <c r="Q51" t="n">
-        <v>0</v>
+        <v>-1800</v>
       </c>
       <c r="R51" t="n">
         <v>-175</v>
@@ -3045,10 +3057,10 @@
       <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="n">
-        <v>-1585</v>
+        <v>-685</v>
       </c>
       <c r="Q52" t="n">
-        <v>0</v>
+        <v>-1800</v>
       </c>
       <c r="R52" t="n">
         <v>425</v>
@@ -3095,10 +3107,10 @@
       <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="n">
-        <v>-1585</v>
+        <v>-685</v>
       </c>
       <c r="Q53" t="n">
-        <v>0</v>
+        <v>-1800</v>
       </c>
       <c r="R53" t="n">
         <v>1025</v>
@@ -3295,10 +3307,10 @@
       <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="n">
+        <v>-900</v>
+      </c>
+      <c r="Q57" t="n">
         <v>0</v>
-      </c>
-      <c r="Q57" t="n">
-        <v>-1380</v>
       </c>
       <c r="R57" t="n">
         <v>-775</v>
@@ -3345,10 +3357,10 @@
       <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="n">
+        <v>-900</v>
+      </c>
+      <c r="Q58" t="n">
         <v>0</v>
-      </c>
-      <c r="Q58" t="n">
-        <v>-1380</v>
       </c>
       <c r="R58" t="n">
         <v>-175</v>
@@ -3395,10 +3407,10 @@
       <c r="N59" t="inlineStr"/>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="n">
+        <v>-900</v>
+      </c>
+      <c r="Q59" t="n">
         <v>0</v>
-      </c>
-      <c r="Q59" t="n">
-        <v>-1380</v>
       </c>
       <c r="R59" t="n">
         <v>425</v>
@@ -3445,10 +3457,10 @@
       <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="n">
+        <v>-900</v>
+      </c>
+      <c r="Q60" t="n">
         <v>0</v>
-      </c>
-      <c r="Q60" t="n">
-        <v>-1380</v>
       </c>
       <c r="R60" t="n">
         <v>1025</v>
@@ -3495,10 +3507,10 @@
       <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="n">
-        <v>600</v>
+        <v>-300</v>
       </c>
       <c r="Q61" t="n">
-        <v>-1380</v>
+        <v>0</v>
       </c>
       <c r="R61" t="n">
         <v>-775</v>
@@ -3545,10 +3557,10 @@
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="n">
-        <v>600</v>
+        <v>-300</v>
       </c>
       <c r="Q62" t="n">
-        <v>-1380</v>
+        <v>0</v>
       </c>
       <c r="R62" t="n">
         <v>-175</v>
@@ -3595,10 +3607,10 @@
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="n">
-        <v>600</v>
+        <v>-300</v>
       </c>
       <c r="Q63" t="n">
-        <v>-1380</v>
+        <v>0</v>
       </c>
       <c r="R63" t="n">
         <v>425</v>
@@ -3645,10 +3657,10 @@
       <c r="N64" t="inlineStr"/>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="n">
-        <v>600</v>
+        <v>-300</v>
       </c>
       <c r="Q64" t="n">
-        <v>-1380</v>
+        <v>0</v>
       </c>
       <c r="R64" t="n">
         <v>1025</v>
@@ -3695,10 +3707,10 @@
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="n">
-        <v>1200</v>
+        <v>300</v>
       </c>
       <c r="Q65" t="n">
-        <v>-1380</v>
+        <v>0</v>
       </c>
       <c r="R65" t="n">
         <v>-775</v>
@@ -3745,10 +3757,10 @@
       <c r="N66" t="inlineStr"/>
       <c r="O66" t="inlineStr"/>
       <c r="P66" t="n">
-        <v>1200</v>
+        <v>300</v>
       </c>
       <c r="Q66" t="n">
-        <v>-1380</v>
+        <v>0</v>
       </c>
       <c r="R66" t="n">
         <v>-175</v>
@@ -3795,10 +3807,10 @@
       <c r="N67" t="inlineStr"/>
       <c r="O67" t="inlineStr"/>
       <c r="P67" t="n">
-        <v>1200</v>
+        <v>300</v>
       </c>
       <c r="Q67" t="n">
-        <v>-1380</v>
+        <v>0</v>
       </c>
       <c r="R67" t="n">
         <v>425</v>
@@ -3845,10 +3857,10 @@
       <c r="N68" t="inlineStr"/>
       <c r="O68" t="inlineStr"/>
       <c r="P68" t="n">
-        <v>1200</v>
+        <v>300</v>
       </c>
       <c r="Q68" t="n">
-        <v>-1380</v>
+        <v>0</v>
       </c>
       <c r="R68" t="n">
         <v>1025</v>
@@ -3895,10 +3907,10 @@
       <c r="N69" t="inlineStr"/>
       <c r="O69" t="inlineStr"/>
       <c r="P69" t="n">
-        <v>1800</v>
+        <v>900</v>
       </c>
       <c r="Q69" t="n">
-        <v>-1380</v>
+        <v>0</v>
       </c>
       <c r="R69" t="n">
         <v>-775</v>
@@ -3945,10 +3957,10 @@
       <c r="N70" t="inlineStr"/>
       <c r="O70" t="inlineStr"/>
       <c r="P70" t="n">
-        <v>1800</v>
+        <v>900</v>
       </c>
       <c r="Q70" t="n">
-        <v>-1380</v>
+        <v>0</v>
       </c>
       <c r="R70" t="n">
         <v>-175</v>
@@ -3995,10 +4007,10 @@
       <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr"/>
       <c r="P71" t="n">
-        <v>1800</v>
+        <v>900</v>
       </c>
       <c r="Q71" t="n">
-        <v>-1380</v>
+        <v>0</v>
       </c>
       <c r="R71" t="n">
         <v>425</v>
@@ -4045,10 +4057,10 @@
       <c r="N72" t="inlineStr"/>
       <c r="O72" t="inlineStr"/>
       <c r="P72" t="n">
-        <v>1800</v>
+        <v>900</v>
       </c>
       <c r="Q72" t="n">
-        <v>-1380</v>
+        <v>0</v>
       </c>
       <c r="R72" t="n">
         <v>1025</v>
@@ -5378,10 +5390,10 @@
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="n">
-        <v>-1330</v>
+        <v>-430</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>-1800</v>
       </c>
       <c r="R5" t="n">
         <v>-375</v>

</xml_diff>

<commit_message>
small fix for annotation
</commit_message>
<xml_diff>
--- a/newui_Greyform/PBU_TERRAHL2(final).xlsx
+++ b/newui_Greyform/PBU_TERRAHL2(final).xlsx
@@ -426,15 +426,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N66"/>
+  <dimension ref="A1:O66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 0</t>
-        </is>
-      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Marking Type</t>
@@ -482,27 +477,32 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Width</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Height</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Orientation</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Diameter</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -532,23 +532,24 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J2" t="n">
         <v>1</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="n">
         <v>2760</v>
       </c>
-      <c r="L2" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>2595</v>
+      </c>
       <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -578,23 +579,24 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J3" t="n">
         <v>1</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="n">
         <v>2760</v>
       </c>
-      <c r="L3" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>2595</v>
+      </c>
       <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -624,23 +626,24 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J4" t="n">
         <v>1</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="n">
         <v>2760</v>
       </c>
-      <c r="L4" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>2595</v>
+      </c>
       <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -670,23 +673,24 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J5" t="n">
         <v>1</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="n">
         <v>2760</v>
       </c>
-      <c r="L5" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>2595</v>
+      </c>
       <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -716,23 +720,24 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J6" t="n">
         <v>1</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="n">
         <v>2760</v>
       </c>
-      <c r="L6" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>2595</v>
+      </c>
       <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -762,23 +767,24 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J7" t="n">
         <v>1</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="n">
         <v>2760</v>
       </c>
-      <c r="L7" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="n">
+        <v>2595</v>
+      </c>
       <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
@@ -808,23 +814,24 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J8" t="n">
         <v>1</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="n">
         <v>2760</v>
       </c>
-      <c r="L8" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>2595</v>
+      </c>
       <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
@@ -854,23 +861,24 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J9" t="n">
         <v>1</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="n">
         <v>2760</v>
       </c>
-      <c r="L9" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>2595</v>
+      </c>
       <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="1" t="n">
         <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -900,23 +908,24 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J10" t="n">
         <v>1</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="n">
         <v>2760</v>
       </c>
-      <c r="L10" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>2595</v>
+      </c>
       <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="1" t="n">
         <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -946,23 +955,24 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J11" t="n">
         <v>1</v>
       </c>
-      <c r="K11" t="n">
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="n">
         <v>2760</v>
       </c>
-      <c r="L11" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>2595</v>
+      </c>
       <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="1" t="n">
         <v>11</v>
       </c>
       <c r="B12" t="inlineStr">
@@ -992,23 +1002,24 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J12" t="n">
         <v>1</v>
       </c>
-      <c r="K12" t="n">
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="n">
         <v>2760</v>
       </c>
-      <c r="L12" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M12" t="inlineStr"/>
+      <c r="M12" t="n">
+        <v>2595</v>
+      </c>
       <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="1" t="n">
         <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
@@ -1038,23 +1049,24 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J13" t="n">
         <v>1</v>
       </c>
-      <c r="K13" t="n">
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="n">
         <v>2760</v>
       </c>
-      <c r="L13" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>2595</v>
+      </c>
       <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="1" t="n">
         <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
@@ -1084,23 +1096,24 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J14" t="n">
         <v>1</v>
       </c>
-      <c r="K14" t="n">
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="n">
         <v>2760</v>
       </c>
-      <c r="L14" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="n">
+        <v>2595</v>
+      </c>
       <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="1" t="n">
         <v>14</v>
       </c>
       <c r="B15" t="inlineStr">
@@ -1130,23 +1143,24 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J15" t="n">
         <v>1</v>
       </c>
-      <c r="K15" t="n">
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="n">
         <v>2760</v>
       </c>
-      <c r="L15" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="n">
+        <v>2595</v>
+      </c>
       <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="1" t="n">
         <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
@@ -1176,23 +1190,24 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J16" t="n">
         <v>1</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="n">
         <v>2760</v>
       </c>
-      <c r="L16" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M16" t="inlineStr"/>
+      <c r="M16" t="n">
+        <v>2595</v>
+      </c>
       <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="1" t="n">
         <v>16</v>
       </c>
       <c r="B17" t="inlineStr">
@@ -1222,23 +1237,24 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J17" t="n">
         <v>1</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
         <v>2760</v>
       </c>
-      <c r="L17" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="n">
+        <v>2595</v>
+      </c>
       <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="1" t="n">
         <v>17</v>
       </c>
       <c r="B18" t="inlineStr">
@@ -1268,23 +1284,24 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J18" t="n">
         <v>1</v>
       </c>
-      <c r="K18" t="n">
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="n">
         <v>1200</v>
       </c>
-      <c r="L18" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M18" t="inlineStr"/>
+      <c r="M18" t="n">
+        <v>2595</v>
+      </c>
       <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="1" t="n">
         <v>18</v>
       </c>
       <c r="B19" t="inlineStr">
@@ -1314,23 +1331,24 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J19" t="n">
         <v>1</v>
       </c>
-      <c r="K19" t="n">
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="n">
         <v>1200</v>
       </c>
-      <c r="L19" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>2595</v>
+      </c>
       <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="1" t="n">
         <v>19</v>
       </c>
       <c r="B20" t="inlineStr">
@@ -1360,23 +1378,24 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J20" t="n">
         <v>1</v>
       </c>
-      <c r="K20" t="n">
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="n">
         <v>1200</v>
       </c>
-      <c r="L20" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>2595</v>
+      </c>
       <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="1" t="n">
         <v>20</v>
       </c>
       <c r="B21" t="inlineStr">
@@ -1406,23 +1425,24 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J21" t="n">
         <v>1</v>
       </c>
-      <c r="K21" t="n">
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="n">
         <v>1200</v>
       </c>
-      <c r="L21" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M21" t="inlineStr"/>
+      <c r="M21" t="n">
+        <v>2595</v>
+      </c>
       <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="1" t="n">
         <v>21</v>
       </c>
       <c r="B22" t="inlineStr">
@@ -1452,23 +1472,24 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J22" t="n">
         <v>1</v>
       </c>
-      <c r="K22" t="n">
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="n">
         <v>1200</v>
       </c>
-      <c r="L22" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M22" t="inlineStr"/>
+      <c r="M22" t="n">
+        <v>2595</v>
+      </c>
       <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="1" t="n">
         <v>22</v>
       </c>
       <c r="B23" t="inlineStr">
@@ -1498,23 +1519,24 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J23" t="n">
         <v>1</v>
       </c>
-      <c r="K23" t="n">
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="n">
         <v>1200</v>
       </c>
-      <c r="L23" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" t="n">
+        <v>2595</v>
+      </c>
       <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" s="1" t="n">
         <v>23</v>
       </c>
       <c r="B24" t="inlineStr">
@@ -1544,23 +1566,24 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J24" t="n">
         <v>1</v>
       </c>
-      <c r="K24" t="n">
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="n">
         <v>960</v>
       </c>
-      <c r="L24" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M24" t="inlineStr"/>
+      <c r="M24" t="n">
+        <v>2595</v>
+      </c>
       <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="n">
+      <c r="A25" s="1" t="n">
         <v>24</v>
       </c>
       <c r="B25" t="inlineStr">
@@ -1590,23 +1613,24 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J25" t="n">
         <v>1</v>
       </c>
-      <c r="K25" t="n">
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="n">
         <v>960</v>
       </c>
-      <c r="L25" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" t="n">
+        <v>2595</v>
+      </c>
       <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" s="1" t="n">
         <v>25</v>
       </c>
       <c r="B26" t="inlineStr">
@@ -1636,23 +1660,24 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J26" t="n">
         <v>1</v>
       </c>
-      <c r="K26" t="n">
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="n">
         <v>960</v>
       </c>
-      <c r="L26" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M26" t="inlineStr"/>
+      <c r="M26" t="n">
+        <v>2595</v>
+      </c>
       <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="n">
+      <c r="A27" s="1" t="n">
         <v>26</v>
       </c>
       <c r="B27" t="inlineStr">
@@ -1682,23 +1707,24 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J27" t="n">
         <v>1</v>
       </c>
-      <c r="K27" t="n">
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="n">
         <v>960</v>
       </c>
-      <c r="L27" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M27" t="inlineStr"/>
+      <c r="M27" t="n">
+        <v>2595</v>
+      </c>
       <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="n">
+      <c r="A28" s="1" t="n">
         <v>27</v>
       </c>
       <c r="B28" t="inlineStr">
@@ -1728,23 +1754,24 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J28" t="n">
         <v>1</v>
       </c>
-      <c r="K28" t="n">
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="n">
         <v>960</v>
       </c>
-      <c r="L28" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M28" t="inlineStr"/>
+      <c r="M28" t="n">
+        <v>2595</v>
+      </c>
       <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="1" t="n">
         <v>28</v>
       </c>
       <c r="B29" t="inlineStr">
@@ -1774,23 +1801,24 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J29" t="n">
         <v>1</v>
       </c>
-      <c r="K29" t="n">
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="n">
         <v>960</v>
       </c>
-      <c r="L29" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M29" t="inlineStr"/>
+      <c r="M29" t="n">
+        <v>2595</v>
+      </c>
       <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="n">
+      <c r="A30" s="1" t="n">
         <v>29</v>
       </c>
       <c r="B30" t="inlineStr">
@@ -1820,23 +1848,24 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J30" t="n">
         <v>1</v>
       </c>
-      <c r="K30" t="n">
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="n">
         <v>960</v>
       </c>
-      <c r="L30" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M30" t="inlineStr"/>
+      <c r="M30" t="n">
+        <v>2595</v>
+      </c>
       <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="1" t="n">
         <v>30</v>
       </c>
       <c r="B31" t="inlineStr">
@@ -1866,23 +1895,24 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J31" t="n">
         <v>1</v>
       </c>
-      <c r="K31" t="n">
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="n">
         <v>960</v>
       </c>
-      <c r="L31" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M31" t="inlineStr"/>
+      <c r="M31" t="n">
+        <v>2595</v>
+      </c>
       <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="n">
+      <c r="A32" s="1" t="n">
         <v>31</v>
       </c>
       <c r="B32" t="inlineStr">
@@ -1912,23 +1942,24 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J32" t="n">
         <v>1</v>
       </c>
-      <c r="K32" t="n">
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="n">
         <v>600</v>
       </c>
-      <c r="L32" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M32" t="inlineStr"/>
+      <c r="M32" t="n">
+        <v>2595</v>
+      </c>
       <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="n">
+      <c r="A33" s="1" t="n">
         <v>32</v>
       </c>
       <c r="B33" t="inlineStr">
@@ -1958,23 +1989,24 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J33" t="n">
         <v>1</v>
       </c>
-      <c r="K33" t="n">
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="n">
         <v>600</v>
       </c>
-      <c r="L33" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M33" t="inlineStr"/>
+      <c r="M33" t="n">
+        <v>2595</v>
+      </c>
       <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="n">
+      <c r="A34" s="1" t="n">
         <v>33</v>
       </c>
       <c r="B34" t="inlineStr">
@@ -2004,23 +2036,24 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J34" t="n">
         <v>1</v>
       </c>
-      <c r="K34" t="n">
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="n">
         <v>600</v>
       </c>
-      <c r="L34" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M34" t="inlineStr"/>
+      <c r="M34" t="n">
+        <v>2595</v>
+      </c>
       <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="n">
+      <c r="A35" s="1" t="n">
         <v>34</v>
       </c>
       <c r="B35" t="inlineStr">
@@ -2050,23 +2083,24 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J35" t="n">
         <v>1</v>
       </c>
-      <c r="K35" t="n">
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="n">
         <v>600</v>
       </c>
-      <c r="L35" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M35" t="inlineStr"/>
+      <c r="M35" t="n">
+        <v>2595</v>
+      </c>
       <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="n">
+      <c r="A36" s="1" t="n">
         <v>35</v>
       </c>
       <c r="B36" t="inlineStr">
@@ -2096,23 +2130,24 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J36" t="n">
         <v>1</v>
       </c>
-      <c r="K36" t="n">
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="n">
         <v>1800</v>
       </c>
-      <c r="L36" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M36" t="inlineStr"/>
+      <c r="M36" t="n">
+        <v>2595</v>
+      </c>
       <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="n">
+      <c r="A37" s="1" t="n">
         <v>36</v>
       </c>
       <c r="B37" t="inlineStr">
@@ -2142,23 +2177,24 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J37" t="n">
         <v>1</v>
       </c>
-      <c r="K37" t="n">
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="n">
         <v>1800</v>
       </c>
-      <c r="L37" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M37" t="inlineStr"/>
+      <c r="M37" t="n">
+        <v>2595</v>
+      </c>
       <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="n">
+      <c r="A38" s="1" t="n">
         <v>37</v>
       </c>
       <c r="B38" t="inlineStr">
@@ -2188,23 +2224,24 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J38" t="n">
         <v>1</v>
       </c>
-      <c r="K38" t="n">
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="n">
         <v>1800</v>
       </c>
-      <c r="L38" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M38" t="inlineStr"/>
+      <c r="M38" t="n">
+        <v>2595</v>
+      </c>
       <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="1" t="n">
         <v>38</v>
       </c>
       <c r="B39" t="inlineStr">
@@ -2234,23 +2271,24 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J39" t="n">
         <v>1</v>
       </c>
-      <c r="K39" t="n">
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="n">
         <v>1800</v>
       </c>
-      <c r="L39" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M39" t="inlineStr"/>
+      <c r="M39" t="n">
+        <v>2595</v>
+      </c>
       <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="1" t="n">
         <v>39</v>
       </c>
       <c r="B40" t="inlineStr">
@@ -2280,23 +2318,24 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J40" t="n">
         <v>1</v>
       </c>
-      <c r="K40" t="n">
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="n">
         <v>1800</v>
       </c>
-      <c r="L40" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M40" t="inlineStr"/>
+      <c r="M40" t="n">
+        <v>2595</v>
+      </c>
       <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="n">
+      <c r="A41" s="1" t="n">
         <v>40</v>
       </c>
       <c r="B41" t="inlineStr">
@@ -2326,23 +2365,24 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J41" t="n">
         <v>1</v>
       </c>
-      <c r="K41" t="n">
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="n">
         <v>1800</v>
       </c>
-      <c r="L41" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M41" t="inlineStr"/>
+      <c r="M41" t="n">
+        <v>2595</v>
+      </c>
       <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" t="n">
+      <c r="A42" s="1" t="n">
         <v>41</v>
       </c>
       <c r="B42" t="inlineStr">
@@ -2372,23 +2412,24 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J42" t="n">
         <v>1</v>
       </c>
-      <c r="K42" t="n">
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="n">
         <v>1800</v>
       </c>
-      <c r="L42" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M42" t="inlineStr"/>
+      <c r="M42" t="n">
+        <v>2595</v>
+      </c>
       <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="1" t="n">
         <v>42</v>
       </c>
       <c r="B43" t="inlineStr">
@@ -2418,23 +2459,24 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J43" t="n">
         <v>1</v>
       </c>
-      <c r="K43" t="n">
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="n">
         <v>1800</v>
       </c>
-      <c r="L43" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M43" t="inlineStr"/>
+      <c r="M43" t="n">
+        <v>2595</v>
+      </c>
       <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="n">
+      <c r="A44" s="1" t="n">
         <v>43</v>
       </c>
       <c r="B44" t="inlineStr">
@@ -2464,23 +2506,24 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J44" t="n">
         <v>1</v>
       </c>
-      <c r="K44" t="n">
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="n">
         <v>1800</v>
       </c>
-      <c r="L44" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M44" t="inlineStr"/>
+      <c r="M44" t="n">
+        <v>2595</v>
+      </c>
       <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="1" t="n">
         <v>44</v>
       </c>
       <c r="B45" t="inlineStr">
@@ -2510,23 +2553,24 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J45" t="n">
         <v>1</v>
       </c>
-      <c r="K45" t="n">
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="n">
         <v>1800</v>
       </c>
-      <c r="L45" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M45" t="inlineStr"/>
+      <c r="M45" t="n">
+        <v>2595</v>
+      </c>
       <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="1" t="n">
         <v>45</v>
       </c>
       <c r="B46" t="inlineStr">
@@ -2556,23 +2600,24 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J46" t="n">
         <v>1</v>
       </c>
-      <c r="K46" t="n">
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="n">
         <v>1800</v>
       </c>
-      <c r="L46" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M46" t="inlineStr"/>
+      <c r="M46" t="n">
+        <v>2595</v>
+      </c>
       <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" t="n">
+      <c r="A47" s="1" t="n">
         <v>46</v>
       </c>
       <c r="B47" t="inlineStr">
@@ -2604,23 +2649,24 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J47" t="n">
         <v>1</v>
       </c>
-      <c r="K47" t="n">
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="n">
         <v>2760</v>
       </c>
-      <c r="L47" t="n">
+      <c r="M47" t="n">
         <v>1800</v>
       </c>
-      <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" t="n">
+      <c r="A48" s="1" t="n">
         <v>47</v>
       </c>
       <c r="B48" t="inlineStr">
@@ -2652,23 +2698,24 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J48" t="n">
         <v>1</v>
       </c>
-      <c r="K48" t="n">
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="n">
         <v>2760</v>
       </c>
-      <c r="L48" t="n">
+      <c r="M48" t="n">
         <v>1800</v>
       </c>
-      <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" t="n">
+      <c r="A49" s="1" t="n">
         <v>48</v>
       </c>
       <c r="B49" t="inlineStr">
@@ -2700,23 +2747,24 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J49" t="n">
         <v>1</v>
       </c>
-      <c r="K49" t="n">
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="n">
         <v>2760</v>
       </c>
-      <c r="L49" t="n">
+      <c r="M49" t="n">
         <v>1800</v>
       </c>
-      <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" t="n">
+      <c r="A50" s="1" t="n">
         <v>49</v>
       </c>
       <c r="B50" t="inlineStr">
@@ -2748,23 +2796,24 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J50" t="n">
         <v>1</v>
       </c>
-      <c r="K50" t="n">
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="n">
         <v>2760</v>
       </c>
-      <c r="L50" t="n">
+      <c r="M50" t="n">
         <v>1800</v>
       </c>
-      <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" t="n">
+      <c r="A51" s="1" t="n">
         <v>50</v>
       </c>
       <c r="B51" t="inlineStr">
@@ -2796,23 +2845,24 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J51" t="n">
         <v>1</v>
       </c>
-      <c r="K51" t="n">
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="n">
         <v>2760</v>
       </c>
-      <c r="L51" t="n">
+      <c r="M51" t="n">
         <v>1800</v>
       </c>
-      <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" t="n">
+      <c r="A52" s="1" t="n">
         <v>51</v>
       </c>
       <c r="B52" t="inlineStr">
@@ -2844,23 +2894,24 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J52" t="n">
         <v>1</v>
       </c>
-      <c r="K52" t="n">
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="n">
         <v>2760</v>
       </c>
-      <c r="L52" t="n">
+      <c r="M52" t="n">
         <v>1800</v>
       </c>
-      <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" t="n">
+      <c r="A53" s="1" t="n">
         <v>52</v>
       </c>
       <c r="B53" t="inlineStr">
@@ -2892,23 +2943,24 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J53" t="n">
         <v>1</v>
       </c>
-      <c r="K53" t="n">
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="n">
         <v>2760</v>
       </c>
-      <c r="L53" t="n">
+      <c r="M53" t="n">
         <v>1800</v>
       </c>
-      <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" t="n">
+      <c r="A54" s="1" t="n">
         <v>53</v>
       </c>
       <c r="B54" t="inlineStr">
@@ -2940,23 +2992,24 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J54" t="n">
         <v>1</v>
       </c>
-      <c r="K54" t="n">
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="n">
         <v>2760</v>
       </c>
-      <c r="L54" t="n">
+      <c r="M54" t="n">
         <v>1800</v>
       </c>
-      <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" t="n">
+      <c r="A55" s="1" t="n">
         <v>54</v>
       </c>
       <c r="B55" t="inlineStr">
@@ -2988,23 +3041,24 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J55" t="n">
         <v>1</v>
       </c>
-      <c r="K55" t="n">
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="n">
         <v>2760</v>
       </c>
-      <c r="L55" t="n">
+      <c r="M55" t="n">
         <v>1800</v>
       </c>
-      <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" t="n">
+      <c r="A56" s="1" t="n">
         <v>55</v>
       </c>
       <c r="B56" t="inlineStr">
@@ -3036,23 +3090,24 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J56" t="n">
         <v>1</v>
       </c>
-      <c r="K56" t="n">
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="n">
         <v>2760</v>
       </c>
-      <c r="L56" t="n">
+      <c r="M56" t="n">
         <v>1800</v>
       </c>
-      <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" t="n">
+      <c r="A57" s="1" t="n">
         <v>56</v>
       </c>
       <c r="B57" t="inlineStr">
@@ -3084,23 +3139,24 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J57" t="n">
         <v>1</v>
       </c>
-      <c r="K57" t="n">
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="n">
         <v>2760</v>
       </c>
-      <c r="L57" t="n">
+      <c r="M57" t="n">
         <v>1800</v>
       </c>
-      <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" t="n">
+      <c r="A58" s="1" t="n">
         <v>57</v>
       </c>
       <c r="B58" t="inlineStr">
@@ -3132,23 +3188,24 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J58" t="n">
         <v>1</v>
       </c>
-      <c r="K58" t="n">
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="n">
         <v>2760</v>
       </c>
-      <c r="L58" t="n">
+      <c r="M58" t="n">
         <v>1800</v>
       </c>
-      <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" t="n">
+      <c r="A59" s="1" t="n">
         <v>58</v>
       </c>
       <c r="B59" t="inlineStr">
@@ -3180,23 +3237,24 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J59" t="n">
         <v>1</v>
       </c>
-      <c r="K59" t="n">
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="n">
         <v>2760</v>
       </c>
-      <c r="L59" t="n">
+      <c r="M59" t="n">
         <v>1800</v>
       </c>
-      <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" t="n">
+      <c r="A60" s="1" t="n">
         <v>59</v>
       </c>
       <c r="B60" t="inlineStr">
@@ -3228,23 +3286,24 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J60" t="n">
         <v>1</v>
       </c>
-      <c r="K60" t="n">
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="n">
         <v>2760</v>
       </c>
-      <c r="L60" t="n">
+      <c r="M60" t="n">
         <v>1800</v>
       </c>
-      <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" t="n">
+      <c r="A61" s="1" t="n">
         <v>60</v>
       </c>
       <c r="B61" t="inlineStr">
@@ -3276,23 +3335,24 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J61" t="n">
         <v>1</v>
       </c>
-      <c r="K61" t="n">
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="n">
         <v>2760</v>
       </c>
-      <c r="L61" t="n">
+      <c r="M61" t="n">
         <v>1800</v>
       </c>
-      <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" t="n">
+      <c r="A62" s="1" t="n">
         <v>61</v>
       </c>
       <c r="B62" t="inlineStr">
@@ -3324,23 +3384,24 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J62" t="n">
         <v>1</v>
       </c>
-      <c r="K62" t="n">
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="n">
         <v>2760</v>
       </c>
-      <c r="L62" t="n">
+      <c r="M62" t="n">
         <v>1800</v>
       </c>
-      <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" t="n">
+      <c r="A63" s="1" t="n">
         <v>62</v>
       </c>
       <c r="B63" t="inlineStr">
@@ -3372,23 +3433,24 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J63" t="n">
         <v>1</v>
       </c>
-      <c r="K63" t="n">
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="n">
         <v>2760</v>
       </c>
-      <c r="L63" t="n">
+      <c r="M63" t="n">
         <v>1800</v>
       </c>
-      <c r="M63" t="inlineStr"/>
       <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" t="n">
+      <c r="A64" s="1" t="n">
         <v>63</v>
       </c>
       <c r="B64" t="inlineStr">
@@ -3420,23 +3482,24 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J64" t="n">
         <v>1</v>
       </c>
-      <c r="K64" t="n">
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="n">
         <v>2760</v>
       </c>
-      <c r="L64" t="n">
+      <c r="M64" t="n">
         <v>1800</v>
       </c>
-      <c r="M64" t="inlineStr"/>
       <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" t="n">
+      <c r="A65" s="1" t="n">
         <v>64</v>
       </c>
       <c r="B65" t="inlineStr">
@@ -3468,23 +3531,24 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J65" t="n">
         <v>1</v>
       </c>
-      <c r="K65" t="n">
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="n">
         <v>2760</v>
       </c>
-      <c r="L65" t="n">
+      <c r="M65" t="n">
         <v>1800</v>
       </c>
-      <c r="M65" t="inlineStr"/>
       <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" t="n">
+      <c r="A66" s="1" t="n">
         <v>65</v>
       </c>
       <c r="B66" t="inlineStr">
@@ -3516,20 +3580,21 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J66" t="n">
         <v>1</v>
       </c>
-      <c r="K66" t="n">
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="n">
         <v>2760</v>
       </c>
-      <c r="L66" t="n">
+      <c r="M66" t="n">
         <v>1800</v>
       </c>
-      <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3542,15 +3607,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 0</t>
-        </is>
-      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Marking Type</t>
@@ -3598,27 +3658,32 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Width</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Height</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Orientation</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Diameter</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="n">
@@ -3646,23 +3711,24 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J2" t="n">
         <v>1</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="n">
         <v>2760</v>
       </c>
-      <c r="L2" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>2595</v>
+      </c>
       <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="B3" t="n">
@@ -3690,23 +3756,24 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J3" t="n">
         <v>1</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="n">
         <v>960</v>
       </c>
-      <c r="L3" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>2595</v>
+      </c>
       <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="B4" t="n">
@@ -3734,23 +3801,24 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J4" t="n">
         <v>1</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="n">
         <v>960</v>
       </c>
-      <c r="L4" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>2595</v>
+      </c>
       <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="B5" t="n">
@@ -3778,23 +3846,24 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J5" t="n">
         <v>1</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="n">
         <v>600</v>
       </c>
-      <c r="L5" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>2595</v>
+      </c>
       <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="B6" t="n">
@@ -3822,23 +3891,24 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J6" t="n">
         <v>1</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="n">
         <v>1800</v>
       </c>
-      <c r="L6" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>2595</v>
+      </c>
       <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
       <c r="B7" t="n">
@@ -3866,23 +3936,24 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J7" t="n">
         <v>1</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="n">
         <v>1800</v>
       </c>
-      <c r="L7" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="n">
+        <v>2595</v>
+      </c>
       <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
       <c r="B8" t="n">
@@ -3910,23 +3981,24 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J8" t="n">
         <v>1</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="n">
         <v>1800</v>
       </c>
-      <c r="L8" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>2595</v>
+      </c>
       <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
       <c r="B9" t="n">
@@ -3954,23 +4026,24 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J9" t="n">
         <v>1</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="n">
         <v>1800</v>
       </c>
-      <c r="L9" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>2595</v>
+      </c>
       <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="1" t="n">
         <v>9</v>
       </c>
       <c r="B10" t="n">
@@ -4000,23 +4073,24 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J10" t="n">
         <v>1</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="n">
         <v>2760</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>1800</v>
       </c>
-      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="1" t="n">
         <v>10</v>
       </c>
       <c r="B11" t="n">
@@ -4046,20 +4120,21 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J11" t="n">
         <v>1</v>
       </c>
-      <c r="K11" t="n">
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="n">
         <v>2760</v>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>1800</v>
       </c>
-      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
changes finalize for the ui
</commit_message>
<xml_diff>
--- a/newui_Greyform/PBU_TERRAHL2(final).xlsx
+++ b/newui_Greyform/PBU_TERRAHL2(final).xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N66"/>
+  <dimension ref="A1:O66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,20 +482,25 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Width</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Height</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Orientation</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Diameter</t>
         </is>
@@ -538,14 +543,15 @@
       <c r="J2" t="n">
         <v>1</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="n">
         <v>2760</v>
       </c>
-      <c r="L2" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>2595</v>
+      </c>
       <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -584,14 +590,15 @@
       <c r="J3" t="n">
         <v>1</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="n">
         <v>2760</v>
       </c>
-      <c r="L3" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>2595</v>
+      </c>
       <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -630,14 +637,15 @@
       <c r="J4" t="n">
         <v>1</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="n">
         <v>2760</v>
       </c>
-      <c r="L4" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>2595</v>
+      </c>
       <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -676,14 +684,15 @@
       <c r="J5" t="n">
         <v>1</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="n">
         <v>2760</v>
       </c>
-      <c r="L5" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>2595</v>
+      </c>
       <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -722,14 +731,15 @@
       <c r="J6" t="n">
         <v>1</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="n">
         <v>2760</v>
       </c>
-      <c r="L6" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>2595</v>
+      </c>
       <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -768,14 +778,15 @@
       <c r="J7" t="n">
         <v>1</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="n">
         <v>2760</v>
       </c>
-      <c r="L7" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="n">
+        <v>2595</v>
+      </c>
       <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -814,14 +825,15 @@
       <c r="J8" t="n">
         <v>1</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="n">
         <v>2760</v>
       </c>
-      <c r="L8" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>2595</v>
+      </c>
       <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -860,14 +872,15 @@
       <c r="J9" t="n">
         <v>1</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="n">
         <v>2760</v>
       </c>
-      <c r="L9" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>2595</v>
+      </c>
       <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -906,14 +919,15 @@
       <c r="J10" t="n">
         <v>1</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="n">
         <v>2760</v>
       </c>
-      <c r="L10" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>2595</v>
+      </c>
       <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -952,14 +966,15 @@
       <c r="J11" t="n">
         <v>1</v>
       </c>
-      <c r="K11" t="n">
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="n">
         <v>2760</v>
       </c>
-      <c r="L11" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>2595</v>
+      </c>
       <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -998,14 +1013,15 @@
       <c r="J12" t="n">
         <v>1</v>
       </c>
-      <c r="K12" t="n">
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="n">
         <v>2760</v>
       </c>
-      <c r="L12" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M12" t="inlineStr"/>
+      <c r="M12" t="n">
+        <v>2595</v>
+      </c>
       <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1044,14 +1060,15 @@
       <c r="J13" t="n">
         <v>1</v>
       </c>
-      <c r="K13" t="n">
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="n">
         <v>2760</v>
       </c>
-      <c r="L13" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>2595</v>
+      </c>
       <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1090,14 +1107,15 @@
       <c r="J14" t="n">
         <v>1</v>
       </c>
-      <c r="K14" t="n">
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="n">
         <v>2760</v>
       </c>
-      <c r="L14" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="n">
+        <v>2595</v>
+      </c>
       <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1136,14 +1154,15 @@
       <c r="J15" t="n">
         <v>1</v>
       </c>
-      <c r="K15" t="n">
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="n">
         <v>2760</v>
       </c>
-      <c r="L15" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="n">
+        <v>2595</v>
+      </c>
       <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1182,14 +1201,15 @@
       <c r="J16" t="n">
         <v>1</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="n">
         <v>2760</v>
       </c>
-      <c r="L16" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M16" t="inlineStr"/>
+      <c r="M16" t="n">
+        <v>2595</v>
+      </c>
       <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1228,14 +1248,15 @@
       <c r="J17" t="n">
         <v>1</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
         <v>2760</v>
       </c>
-      <c r="L17" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="n">
+        <v>2595</v>
+      </c>
       <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1274,14 +1295,15 @@
       <c r="J18" t="n">
         <v>1</v>
       </c>
-      <c r="K18" t="n">
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="n">
         <v>1200</v>
       </c>
-      <c r="L18" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M18" t="inlineStr"/>
+      <c r="M18" t="n">
+        <v>2595</v>
+      </c>
       <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1320,14 +1342,15 @@
       <c r="J19" t="n">
         <v>1</v>
       </c>
-      <c r="K19" t="n">
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="n">
         <v>1200</v>
       </c>
-      <c r="L19" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>2595</v>
+      </c>
       <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1366,14 +1389,15 @@
       <c r="J20" t="n">
         <v>1</v>
       </c>
-      <c r="K20" t="n">
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="n">
         <v>1200</v>
       </c>
-      <c r="L20" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>2595</v>
+      </c>
       <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1412,14 +1436,15 @@
       <c r="J21" t="n">
         <v>1</v>
       </c>
-      <c r="K21" t="n">
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="n">
         <v>1200</v>
       </c>
-      <c r="L21" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M21" t="inlineStr"/>
+      <c r="M21" t="n">
+        <v>2595</v>
+      </c>
       <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1458,14 +1483,15 @@
       <c r="J22" t="n">
         <v>1</v>
       </c>
-      <c r="K22" t="n">
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="n">
         <v>1200</v>
       </c>
-      <c r="L22" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M22" t="inlineStr"/>
+      <c r="M22" t="n">
+        <v>2595</v>
+      </c>
       <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1504,14 +1530,15 @@
       <c r="J23" t="n">
         <v>1</v>
       </c>
-      <c r="K23" t="n">
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="n">
         <v>1200</v>
       </c>
-      <c r="L23" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" t="n">
+        <v>2595</v>
+      </c>
       <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1550,14 +1577,15 @@
       <c r="J24" t="n">
         <v>1</v>
       </c>
-      <c r="K24" t="n">
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="n">
         <v>960</v>
       </c>
-      <c r="L24" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M24" t="inlineStr"/>
+      <c r="M24" t="n">
+        <v>2595</v>
+      </c>
       <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1596,14 +1624,15 @@
       <c r="J25" t="n">
         <v>1</v>
       </c>
-      <c r="K25" t="n">
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="n">
         <v>960</v>
       </c>
-      <c r="L25" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" t="n">
+        <v>2595</v>
+      </c>
       <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1642,14 +1671,15 @@
       <c r="J26" t="n">
         <v>1</v>
       </c>
-      <c r="K26" t="n">
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="n">
         <v>960</v>
       </c>
-      <c r="L26" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M26" t="inlineStr"/>
+      <c r="M26" t="n">
+        <v>2595</v>
+      </c>
       <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1688,14 +1718,15 @@
       <c r="J27" t="n">
         <v>1</v>
       </c>
-      <c r="K27" t="n">
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="n">
         <v>960</v>
       </c>
-      <c r="L27" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M27" t="inlineStr"/>
+      <c r="M27" t="n">
+        <v>2595</v>
+      </c>
       <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1734,14 +1765,15 @@
       <c r="J28" t="n">
         <v>1</v>
       </c>
-      <c r="K28" t="n">
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="n">
         <v>960</v>
       </c>
-      <c r="L28" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M28" t="inlineStr"/>
+      <c r="M28" t="n">
+        <v>2595</v>
+      </c>
       <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1780,14 +1812,15 @@
       <c r="J29" t="n">
         <v>1</v>
       </c>
-      <c r="K29" t="n">
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="n">
         <v>960</v>
       </c>
-      <c r="L29" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M29" t="inlineStr"/>
+      <c r="M29" t="n">
+        <v>2595</v>
+      </c>
       <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1826,14 +1859,15 @@
       <c r="J30" t="n">
         <v>1</v>
       </c>
-      <c r="K30" t="n">
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="n">
         <v>960</v>
       </c>
-      <c r="L30" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M30" t="inlineStr"/>
+      <c r="M30" t="n">
+        <v>2595</v>
+      </c>
       <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1872,14 +1906,15 @@
       <c r="J31" t="n">
         <v>1</v>
       </c>
-      <c r="K31" t="n">
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="n">
         <v>960</v>
       </c>
-      <c r="L31" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M31" t="inlineStr"/>
+      <c r="M31" t="n">
+        <v>2595</v>
+      </c>
       <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1918,14 +1953,15 @@
       <c r="J32" t="n">
         <v>1</v>
       </c>
-      <c r="K32" t="n">
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="n">
         <v>600</v>
       </c>
-      <c r="L32" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M32" t="inlineStr"/>
+      <c r="M32" t="n">
+        <v>2595</v>
+      </c>
       <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1964,14 +2000,15 @@
       <c r="J33" t="n">
         <v>1</v>
       </c>
-      <c r="K33" t="n">
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="n">
         <v>600</v>
       </c>
-      <c r="L33" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M33" t="inlineStr"/>
+      <c r="M33" t="n">
+        <v>2595</v>
+      </c>
       <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2010,14 +2047,15 @@
       <c r="J34" t="n">
         <v>1</v>
       </c>
-      <c r="K34" t="n">
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="n">
         <v>600</v>
       </c>
-      <c r="L34" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M34" t="inlineStr"/>
+      <c r="M34" t="n">
+        <v>2595</v>
+      </c>
       <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2056,14 +2094,15 @@
       <c r="J35" t="n">
         <v>1</v>
       </c>
-      <c r="K35" t="n">
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="n">
         <v>600</v>
       </c>
-      <c r="L35" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M35" t="inlineStr"/>
+      <c r="M35" t="n">
+        <v>2595</v>
+      </c>
       <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2102,14 +2141,15 @@
       <c r="J36" t="n">
         <v>1</v>
       </c>
-      <c r="K36" t="n">
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="n">
         <v>1800</v>
       </c>
-      <c r="L36" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M36" t="inlineStr"/>
+      <c r="M36" t="n">
+        <v>2595</v>
+      </c>
       <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2148,14 +2188,15 @@
       <c r="J37" t="n">
         <v>1</v>
       </c>
-      <c r="K37" t="n">
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="n">
         <v>1800</v>
       </c>
-      <c r="L37" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M37" t="inlineStr"/>
+      <c r="M37" t="n">
+        <v>2595</v>
+      </c>
       <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2194,14 +2235,15 @@
       <c r="J38" t="n">
         <v>1</v>
       </c>
-      <c r="K38" t="n">
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="n">
         <v>1800</v>
       </c>
-      <c r="L38" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M38" t="inlineStr"/>
+      <c r="M38" t="n">
+        <v>2595</v>
+      </c>
       <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2240,14 +2282,15 @@
       <c r="J39" t="n">
         <v>1</v>
       </c>
-      <c r="K39" t="n">
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="n">
         <v>1800</v>
       </c>
-      <c r="L39" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M39" t="inlineStr"/>
+      <c r="M39" t="n">
+        <v>2595</v>
+      </c>
       <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2286,14 +2329,15 @@
       <c r="J40" t="n">
         <v>1</v>
       </c>
-      <c r="K40" t="n">
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="n">
         <v>1800</v>
       </c>
-      <c r="L40" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M40" t="inlineStr"/>
+      <c r="M40" t="n">
+        <v>2595</v>
+      </c>
       <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2332,14 +2376,15 @@
       <c r="J41" t="n">
         <v>1</v>
       </c>
-      <c r="K41" t="n">
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="n">
         <v>1800</v>
       </c>
-      <c r="L41" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M41" t="inlineStr"/>
+      <c r="M41" t="n">
+        <v>2595</v>
+      </c>
       <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2378,14 +2423,15 @@
       <c r="J42" t="n">
         <v>1</v>
       </c>
-      <c r="K42" t="n">
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="n">
         <v>1800</v>
       </c>
-      <c r="L42" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M42" t="inlineStr"/>
+      <c r="M42" t="n">
+        <v>2595</v>
+      </c>
       <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2424,14 +2470,15 @@
       <c r="J43" t="n">
         <v>1</v>
       </c>
-      <c r="K43" t="n">
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="n">
         <v>1800</v>
       </c>
-      <c r="L43" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M43" t="inlineStr"/>
+      <c r="M43" t="n">
+        <v>2595</v>
+      </c>
       <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2470,14 +2517,15 @@
       <c r="J44" t="n">
         <v>1</v>
       </c>
-      <c r="K44" t="n">
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="n">
         <v>1800</v>
       </c>
-      <c r="L44" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M44" t="inlineStr"/>
+      <c r="M44" t="n">
+        <v>2595</v>
+      </c>
       <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2516,14 +2564,15 @@
       <c r="J45" t="n">
         <v>1</v>
       </c>
-      <c r="K45" t="n">
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="n">
         <v>1800</v>
       </c>
-      <c r="L45" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M45" t="inlineStr"/>
+      <c r="M45" t="n">
+        <v>2595</v>
+      </c>
       <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2562,14 +2611,15 @@
       <c r="J46" t="n">
         <v>1</v>
       </c>
-      <c r="K46" t="n">
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="n">
         <v>1800</v>
       </c>
-      <c r="L46" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M46" t="inlineStr"/>
+      <c r="M46" t="n">
+        <v>2595</v>
+      </c>
       <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2610,14 +2660,15 @@
       <c r="J47" t="n">
         <v>1</v>
       </c>
-      <c r="K47" t="n">
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="n">
         <v>2760</v>
       </c>
-      <c r="L47" t="n">
+      <c r="M47" t="n">
         <v>1800</v>
       </c>
-      <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2658,14 +2709,15 @@
       <c r="J48" t="n">
         <v>1</v>
       </c>
-      <c r="K48" t="n">
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="n">
         <v>2760</v>
       </c>
-      <c r="L48" t="n">
+      <c r="M48" t="n">
         <v>1800</v>
       </c>
-      <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2706,14 +2758,15 @@
       <c r="J49" t="n">
         <v>1</v>
       </c>
-      <c r="K49" t="n">
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="n">
         <v>2760</v>
       </c>
-      <c r="L49" t="n">
+      <c r="M49" t="n">
         <v>1800</v>
       </c>
-      <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2754,14 +2807,15 @@
       <c r="J50" t="n">
         <v>1</v>
       </c>
-      <c r="K50" t="n">
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="n">
         <v>2760</v>
       </c>
-      <c r="L50" t="n">
+      <c r="M50" t="n">
         <v>1800</v>
       </c>
-      <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2802,14 +2856,15 @@
       <c r="J51" t="n">
         <v>1</v>
       </c>
-      <c r="K51" t="n">
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="n">
         <v>2760</v>
       </c>
-      <c r="L51" t="n">
+      <c r="M51" t="n">
         <v>1800</v>
       </c>
-      <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2850,14 +2905,15 @@
       <c r="J52" t="n">
         <v>1</v>
       </c>
-      <c r="K52" t="n">
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="n">
         <v>2760</v>
       </c>
-      <c r="L52" t="n">
+      <c r="M52" t="n">
         <v>1800</v>
       </c>
-      <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2898,14 +2954,15 @@
       <c r="J53" t="n">
         <v>1</v>
       </c>
-      <c r="K53" t="n">
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="n">
         <v>2760</v>
       </c>
-      <c r="L53" t="n">
+      <c r="M53" t="n">
         <v>1800</v>
       </c>
-      <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2946,14 +3003,15 @@
       <c r="J54" t="n">
         <v>1</v>
       </c>
-      <c r="K54" t="n">
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="n">
         <v>2760</v>
       </c>
-      <c r="L54" t="n">
+      <c r="M54" t="n">
         <v>1800</v>
       </c>
-      <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2994,14 +3052,15 @@
       <c r="J55" t="n">
         <v>1</v>
       </c>
-      <c r="K55" t="n">
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="n">
         <v>2760</v>
       </c>
-      <c r="L55" t="n">
+      <c r="M55" t="n">
         <v>1800</v>
       </c>
-      <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -3042,14 +3101,15 @@
       <c r="J56" t="n">
         <v>1</v>
       </c>
-      <c r="K56" t="n">
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="n">
         <v>2760</v>
       </c>
-      <c r="L56" t="n">
+      <c r="M56" t="n">
         <v>1800</v>
       </c>
-      <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -3090,14 +3150,15 @@
       <c r="J57" t="n">
         <v>1</v>
       </c>
-      <c r="K57" t="n">
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="n">
         <v>2760</v>
       </c>
-      <c r="L57" t="n">
+      <c r="M57" t="n">
         <v>1800</v>
       </c>
-      <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3138,14 +3199,15 @@
       <c r="J58" t="n">
         <v>1</v>
       </c>
-      <c r="K58" t="n">
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="n">
         <v>2760</v>
       </c>
-      <c r="L58" t="n">
+      <c r="M58" t="n">
         <v>1800</v>
       </c>
-      <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -3186,14 +3248,15 @@
       <c r="J59" t="n">
         <v>1</v>
       </c>
-      <c r="K59" t="n">
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="n">
         <v>2760</v>
       </c>
-      <c r="L59" t="n">
+      <c r="M59" t="n">
         <v>1800</v>
       </c>
-      <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3234,14 +3297,15 @@
       <c r="J60" t="n">
         <v>1</v>
       </c>
-      <c r="K60" t="n">
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="n">
         <v>2760</v>
       </c>
-      <c r="L60" t="n">
+      <c r="M60" t="n">
         <v>1800</v>
       </c>
-      <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3282,14 +3346,15 @@
       <c r="J61" t="n">
         <v>1</v>
       </c>
-      <c r="K61" t="n">
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="n">
         <v>2760</v>
       </c>
-      <c r="L61" t="n">
+      <c r="M61" t="n">
         <v>1800</v>
       </c>
-      <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -3330,14 +3395,15 @@
       <c r="J62" t="n">
         <v>1</v>
       </c>
-      <c r="K62" t="n">
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="n">
         <v>2760</v>
       </c>
-      <c r="L62" t="n">
+      <c r="M62" t="n">
         <v>1800</v>
       </c>
-      <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3378,14 +3444,15 @@
       <c r="J63" t="n">
         <v>1</v>
       </c>
-      <c r="K63" t="n">
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="n">
         <v>2760</v>
       </c>
-      <c r="L63" t="n">
+      <c r="M63" t="n">
         <v>1800</v>
       </c>
-      <c r="M63" t="inlineStr"/>
       <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3426,14 +3493,15 @@
       <c r="J64" t="n">
         <v>1</v>
       </c>
-      <c r="K64" t="n">
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="n">
         <v>2760</v>
       </c>
-      <c r="L64" t="n">
+      <c r="M64" t="n">
         <v>1800</v>
       </c>
-      <c r="M64" t="inlineStr"/>
       <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3474,14 +3542,15 @@
       <c r="J65" t="n">
         <v>1</v>
       </c>
-      <c r="K65" t="n">
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="n">
         <v>2760</v>
       </c>
-      <c r="L65" t="n">
+      <c r="M65" t="n">
         <v>1800</v>
       </c>
-      <c r="M65" t="inlineStr"/>
       <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3522,14 +3591,15 @@
       <c r="J66" t="n">
         <v>1</v>
       </c>
-      <c r="K66" t="n">
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="n">
         <v>2760</v>
       </c>
-      <c r="L66" t="n">
+      <c r="M66" t="n">
         <v>1800</v>
       </c>
-      <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3542,7 +3612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3598,20 +3668,25 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Width</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Height</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Orientation</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Diameter</t>
         </is>
@@ -3652,14 +3727,15 @@
       <c r="J2" t="n">
         <v>1</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="n">
         <v>2760</v>
       </c>
-      <c r="L2" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>2595</v>
+      </c>
       <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -3696,14 +3772,15 @@
       <c r="J3" t="n">
         <v>1</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="n">
         <v>960</v>
       </c>
-      <c r="L3" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>2595</v>
+      </c>
       <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -3740,14 +3817,15 @@
       <c r="J4" t="n">
         <v>1</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="n">
         <v>960</v>
       </c>
-      <c r="L4" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>2595</v>
+      </c>
       <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -3784,14 +3862,15 @@
       <c r="J5" t="n">
         <v>1</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="n">
         <v>600</v>
       </c>
-      <c r="L5" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>2595</v>
+      </c>
       <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -3828,14 +3907,15 @@
       <c r="J6" t="n">
         <v>1</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="n">
         <v>1800</v>
       </c>
-      <c r="L6" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>2595</v>
+      </c>
       <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -3872,14 +3952,15 @@
       <c r="J7" t="n">
         <v>1</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="n">
         <v>1800</v>
       </c>
-      <c r="L7" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="n">
+        <v>2595</v>
+      </c>
       <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -3916,14 +3997,15 @@
       <c r="J8" t="n">
         <v>1</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="n">
         <v>1800</v>
       </c>
-      <c r="L8" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>2595</v>
+      </c>
       <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -3960,14 +4042,15 @@
       <c r="J9" t="n">
         <v>1</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="n">
         <v>1800</v>
       </c>
-      <c r="L9" t="n">
-        <v>2595</v>
-      </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>2595</v>
+      </c>
       <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -4006,14 +4089,15 @@
       <c r="J10" t="n">
         <v>1</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="n">
         <v>2760</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>1800</v>
       </c>
-      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -4052,14 +4136,15 @@
       <c r="J11" t="n">
         <v>1</v>
       </c>
-      <c r="K11" t="n">
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="n">
         <v>2760</v>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>1800</v>
       </c>
-      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>